<commit_message>
feat(config): G03-P3-B2 author universe topology
</commit_message>
<xml_diff>
--- a/config/generated/templates/Universe.xlsx
+++ b/config/generated/templates/Universe.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="263">
   <si>
     <t>@table</t>
   </si>
@@ -248,7 +248,7 @@
     <t>list</t>
   </si>
   <si>
-    <t>28b51f23ed1c8123</t>
+    <t>53e48fcfb13ef795</t>
   </si>
   <si>
     <t>difficulty_id</t>
@@ -263,7 +263,7 @@
     <t>source_monster_id</t>
   </si>
   <si>
-    <t>enemy_variant_id</t>
+    <t>enemy_variant_stable_key</t>
   </si>
   <si>
     <t>level</t>
@@ -273,9 +273,6 @@
   </si>
   <si>
     <t>enum&lt;UniverseEnemyRole&gt;</t>
-  </si>
-  <si>
-    <t>ref&lt;EnemyVariant.id&gt;</t>
   </si>
   <si>
     <t>range=1..100</t>
@@ -1505,7 +1502,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1529,7 +1526,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -1543,7 +1540,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>37</v>
@@ -1558,7 +1555,7 @@
         <v>40</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1572,7 +1569,7 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>37</v>
@@ -1587,7 +1584,7 @@
         <v>40</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1717,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1739,7 +1736,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -1747,13 +1744,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1761,13 +1758,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1775,7 +1772,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -1804,7 +1801,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>26</v>
@@ -1852,7 +1849,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1876,7 +1873,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -1890,19 +1887,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>133</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>37</v>
@@ -1917,13 +1914,13 @@
         <v>40</v>
       </c>
       <c r="M2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -1937,19 +1934,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>132</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>37</v>
@@ -1964,13 +1961,13 @@
         <v>40</v>
       </c>
       <c r="M3" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="O3" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -1984,10 +1981,10 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>21</v>
@@ -2080,7 +2077,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>27</v>
@@ -2101,7 +2098,7 @@
         <v>46</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>45</v>
@@ -2163,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2185,7 +2182,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2193,13 +2190,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2207,13 +2204,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2221,7 +2218,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -2250,7 +2247,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -2297,7 +2294,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2321,7 +2318,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="24" customHeight="1">
@@ -2335,10 +2332,10 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>37</v>
@@ -2353,19 +2350,19 @@
         <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -2379,10 +2376,10 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>37</v>
@@ -2397,19 +2394,19 @@
         <v>40</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="M3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K3" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="M3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>150</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -2423,7 +2420,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>21</v>
@@ -2512,7 +2509,7 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>45</v>
@@ -2527,10 +2524,10 @@
         <v>46</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>26</v>
@@ -2591,7 +2588,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2613,7 +2610,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2621,13 +2618,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2635,13 +2632,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2649,13 +2646,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2678,7 +2675,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5"/>
     </row>
@@ -2721,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2745,7 +2742,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -2759,16 +2756,16 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>73</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>136</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>37</v>
@@ -2794,16 +2791,16 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>73</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>37</v>
@@ -2829,7 +2826,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>21</v>
@@ -2896,23 +2893,23 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>45</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>46</v>
@@ -2967,7 +2964,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2989,7 +2986,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2997,13 +2994,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3011,13 +3008,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3025,7 +3022,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -3054,7 +3051,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -3099,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3123,7 +3120,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
@@ -3137,10 +3134,10 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>170</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>171</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>37</v>
@@ -3155,13 +3152,13 @@
         <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -3175,10 +3172,10 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>171</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>37</v>
@@ -3193,13 +3190,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -3289,10 +3286,10 @@
         <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>45</v>
@@ -3307,10 +3304,10 @@
         <v>46</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>26</v>
@@ -3370,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3394,7 +3391,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -3408,28 +3405,28 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="K2" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>37</v>
@@ -3455,28 +3452,28 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>181</v>
-      </c>
       <c r="K3" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -3502,22 +3499,22 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>183</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>60</v>
       </c>
       <c r="G4" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>185</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>22</v>
@@ -3593,7 +3590,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -3607,13 +3604,13 @@
         <v>27</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>46</v>
@@ -3920,7 +3917,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3942,7 +3939,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -3950,13 +3947,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3964,13 +3961,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3978,7 +3975,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4007,7 +4004,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -4049,7 +4046,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4073,7 +4070,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4087,13 +4084,13 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>193</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>37</v>
@@ -4119,13 +4116,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>37</v>
@@ -4157,7 +4154,7 @@
         <v>59</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>22</v>
@@ -4212,13 +4209,13 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
@@ -4281,7 +4278,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4305,7 +4302,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -4319,16 +4316,16 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>37</v>
@@ -4354,16 +4351,16 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>198</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>199</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>37</v>
@@ -4389,7 +4386,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
@@ -4456,23 +4453,23 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>31</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>46</v>
@@ -4530,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4554,7 +4551,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -4568,28 +4565,28 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>210</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>211</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>37</v>
@@ -4615,28 +4612,28 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="K3" s="5" t="s">
         <v>210</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>211</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -4662,7 +4659,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>59</v>
@@ -4757,11 +4754,11 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>29</v>
@@ -4776,10 +4773,10 @@
         <v>29</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>46</v>
@@ -4833,7 +4830,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4855,7 +4852,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4863,7 +4860,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -4872,7 +4869,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -4880,7 +4877,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -4889,7 +4886,7 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4897,7 +4894,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4932,13 +4929,13 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>31</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -4980,7 +4977,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5002,7 +4999,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5010,28 +5007,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5039,28 +5036,28 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5068,7 +5065,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5127,22 +5124,22 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I6" s="5"/>
     </row>
@@ -5191,7 +5188,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5215,7 +5212,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
@@ -5232,16 +5229,16 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>37</v>
@@ -5270,16 +5267,16 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="H3" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>37</v>
@@ -5305,7 +5302,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>60</v>
@@ -5378,20 +5375,20 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>46</v>
@@ -5445,7 +5442,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5467,7 +5464,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5475,16 +5472,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>235</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5492,16 +5489,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5509,7 +5506,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5544,7 +5541,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>26</v>
@@ -5594,7 +5591,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5618,7 +5615,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
@@ -5632,22 +5629,22 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>244</v>
-      </c>
       <c r="I2" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>37</v>
@@ -5673,22 +5670,22 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>244</v>
-      </c>
       <c r="I3" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>37</v>
@@ -5714,10 +5711,10 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>22</v>
@@ -5793,7 +5790,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -5804,16 +5801,16 @@
         <v>45</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>46</v>
@@ -5872,7 +5869,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5894,7 +5891,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5902,13 +5899,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5916,13 +5913,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5930,13 +5927,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -5959,7 +5956,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5"/>
     </row>
@@ -6252,7 +6249,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6274,7 +6271,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6282,16 +6279,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6299,16 +6296,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6316,7 +6313,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6351,7 +6348,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -6400,7 +6397,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6422,7 +6419,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6430,7 +6427,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6439,16 +6436,16 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6456,7 +6453,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6465,16 +6462,16 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>258</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6482,22 +6479,22 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>60</v>
@@ -6535,11 +6532,11 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>27</v>
@@ -6592,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6614,7 +6611,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6622,13 +6619,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6636,13 +6633,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6650,7 +6647,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6679,7 +6676,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -6714,7 +6711,7 @@
     <col min="3" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="23.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" style="5" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6811,7 +6808,7 @@
         <v>22</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>76</v>
+        <v>22</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>21</v>
@@ -6846,13 +6843,15 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="5"/>
+      <c r="F6" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G6" s="5" t="s">
         <v>62</v>
       </c>
@@ -6904,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6928,7 +6927,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -6942,16 +6941,16 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>37</v>
@@ -6977,16 +6976,16 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>82</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>37</v>
@@ -7015,13 +7014,13 @@
         <v>21</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>22</v>
@@ -7156,7 +7155,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7180,7 +7179,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7194,19 +7193,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7220,19 +7219,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7252,7 +7251,7 @@
         <v>21</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>21</v>
@@ -7298,17 +7297,17 @@
         <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -7369,7 +7368,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7391,7 +7390,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7399,13 +7398,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7413,13 +7412,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7427,13 +7426,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7456,7 +7455,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="5"/>
     </row>
@@ -7498,7 +7497,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7522,7 +7521,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7536,19 +7535,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7562,19 +7561,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7588,19 +7587,19 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7650,7 +7649,7 @@
         <v>27</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -7695,7 +7694,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7717,7 +7716,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7725,22 +7724,22 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>52</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7748,22 +7747,22 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>52</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7771,7 +7770,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -7783,10 +7782,10 @@
         <v>22</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7818,7 +7817,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
feat(config): G03-P3-B3 author paths and blessings
</commit_message>
<xml_diff>
--- a/config/generated/templates/Universe.xlsx
+++ b/config/generated/templates/Universe.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="264">
   <si>
     <t>@table</t>
   </si>
@@ -434,7 +434,7 @@
     <t>UniverseResonance</t>
   </si>
   <si>
-    <t>bc6b5653d147c6d4</t>
+    <t>d6e09ab66ac62a17</t>
   </si>
   <si>
     <t>threshold</t>
@@ -458,6 +458,9 @@
     <t>enum&lt;UniverseResonanceKind&gt;</t>
   </si>
   <si>
+    <t>optional&lt;list&lt;string&gt;&gt;</t>
+  </si>
+  <si>
     <t>range=0..18</t>
   </si>
   <si>
@@ -485,7 +488,7 @@
     <t>UniverseBlessing</t>
   </si>
   <si>
-    <t>1f61debc230f1f30</t>
+    <t>8479cfe550c6647c</t>
   </si>
   <si>
     <t>rarity</t>
@@ -506,13 +509,13 @@
     <t>UniverseBlessingPrerequisite</t>
   </si>
   <si>
-    <t>b06533588ebe3a00</t>
+    <t>64ce040b66e5c5c9</t>
   </si>
   <si>
     <t>blessing_id</t>
   </si>
   <si>
-    <t>prerequisite_blessing_id</t>
+    <t>prerequisite_stable_key</t>
   </si>
   <si>
     <t>ref&lt;UniverseBlessing.id&gt;</t>
@@ -521,15 +524,15 @@
     <t>range=1..32</t>
   </si>
   <si>
+    <t>length=1..180</t>
+  </si>
+  <si>
     <t>UniverseBlessingLevel</t>
   </si>
   <si>
     <t>1ff35b47c14c1df5</t>
   </si>
   <si>
-    <t>length=1..180</t>
-  </si>
-  <si>
     <t>range=1..2</t>
   </si>
   <si>
@@ -551,7 +554,7 @@
     <t>UniverseCurio</t>
   </si>
   <si>
-    <t>1169340e9b01e3ab</t>
+    <t>3ccdf0099f816b1f</t>
   </si>
   <si>
     <t>initial_state_stable_key</t>
@@ -617,7 +620,7 @@
     <t>UniverseOccurrence</t>
   </si>
   <si>
-    <t>0f7129e626a92ac7</t>
+    <t>c2a883f31a436270</t>
   </si>
   <si>
     <t>choice_graph_stable_key</t>
@@ -629,7 +632,7 @@
     <t>UniverseOccurrenceVariant</t>
   </si>
   <si>
-    <t>608a789398fb18a1</t>
+    <t>8b8fced2c6c96f4e</t>
   </si>
   <si>
     <t>occurrence_id</t>
@@ -656,7 +659,7 @@
     <t>UniverseOccurrenceChoice</t>
   </si>
   <si>
-    <t>96db64945cd87f18</t>
+    <t>269b40608465c555</t>
   </si>
   <si>
     <t>variant_id</t>
@@ -689,7 +692,7 @@
     <t>UniverseOccurrenceCost</t>
   </si>
   <si>
-    <t>301247fe677849bc</t>
+    <t>99988f4717345da5</t>
   </si>
   <si>
     <t>choice_id</t>
@@ -704,7 +707,7 @@
     <t>UniverseOccurrenceOutcome</t>
   </si>
   <si>
-    <t>0c0601c1ace06ad1</t>
+    <t>f9a05ceb8a2b9e0d</t>
   </si>
   <si>
     <t>kinds</t>
@@ -761,7 +764,7 @@
     <t>UniverseAbilityTreeNode</t>
   </si>
   <si>
-    <t>d7aeb4699c4aa704</t>
+    <t>734569068a3ba709</t>
   </si>
   <si>
     <t>important</t>
@@ -1839,7 +1842,8 @@
     <col min="7" max="7" width="18.7109375" style="5" customWidth="1"/>
     <col min="8" max="8" width="22.7109375" style="5" customWidth="1"/>
     <col min="9" max="11" width="12.7109375" style="5" customWidth="1"/>
-    <col min="12" max="13" width="13.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="18.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="15.7109375" style="5" customWidth="1"/>
   </cols>
@@ -2008,7 +2012,7 @@
         <v>22</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>22</v>
@@ -2077,7 +2081,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>27</v>
@@ -2098,7 +2102,7 @@
         <v>46</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>45</v>
@@ -2160,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2182,7 +2186,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2190,13 +2194,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2204,13 +2208,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2218,7 +2222,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -2247,7 +2251,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -2282,8 +2286,7 @@
     <col min="4" max="4" width="20.7109375" style="5" customWidth="1"/>
     <col min="5" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="11" width="22.7109375" style="5" customWidth="1"/>
     <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="28.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="31.7109375" style="5" customWidth="1"/>
@@ -2294,7 +2297,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2318,7 +2321,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="24" customHeight="1">
@@ -2335,7 +2338,7 @@
         <v>124</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>37</v>
@@ -2350,7 +2353,7 @@
         <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>133</v>
@@ -2359,10 +2362,10 @@
         <v>135</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -2379,7 +2382,7 @@
         <v>124</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>37</v>
@@ -2394,7 +2397,7 @@
         <v>40</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>133</v>
@@ -2403,10 +2406,10 @@
         <v>135</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -2438,10 +2441,10 @@
         <v>22</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>22</v>
@@ -2509,7 +2512,7 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>45</v>
@@ -2524,10 +2527,10 @@
         <v>46</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>26</v>
@@ -2580,7 +2583,7 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" style="5" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -2588,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2610,7 +2613,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2618,13 +2621,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2632,13 +2635,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2646,13 +2649,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>156</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2675,9 +2678,11 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="D6" s="5"/>
+        <v>158</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -2718,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2742,7 +2747,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -2756,7 +2761,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>73</v>
@@ -2791,7 +2796,7 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>73</v>
@@ -2826,7 +2831,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>21</v>
@@ -2893,23 +2898,23 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>45</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>46</v>
@@ -2964,7 +2969,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2986,7 +2991,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2994,13 +2999,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3008,13 +3013,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3022,7 +3027,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -3051,7 +3056,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -3087,7 +3092,7 @@
     <col min="5" max="5" width="14.7109375" style="5" customWidth="1"/>
     <col min="6" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="11" width="12.7109375" style="5" customWidth="1"/>
+    <col min="10" max="11" width="22.7109375" style="5" customWidth="1"/>
     <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3096,7 +3101,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3120,7 +3125,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
@@ -3134,10 +3139,10 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>37</v>
@@ -3152,10 +3157,10 @@
         <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>135</v>
@@ -3172,10 +3177,10 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>37</v>
@@ -3190,10 +3195,10 @@
         <v>40</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>135</v>
@@ -3228,10 +3233,10 @@
         <v>22</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>22</v>
@@ -3286,7 +3291,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>93</v>
@@ -3304,10 +3309,10 @@
         <v>46</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>26</v>
@@ -3367,7 +3372,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3391,7 +3396,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -3405,25 +3410,25 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>135</v>
@@ -3452,25 +3457,25 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>135</v>
@@ -3499,22 +3504,22 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>60</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>22</v>
@@ -3590,7 +3595,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -3604,13 +3609,13 @@
         <v>27</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>46</v>
@@ -3917,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3939,7 +3944,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -3947,13 +3952,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3961,13 +3966,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3975,7 +3980,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4004,7 +4009,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -4037,7 +4042,8 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="23.7109375" style="5" customWidth="1"/>
-    <col min="5" max="9" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="5" customWidth="1"/>
+    <col min="6" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4046,7 +4052,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4070,7 +4076,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4084,13 +4090,13 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>37</v>
@@ -4116,13 +4122,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>37</v>
@@ -4151,7 +4157,7 @@
         <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>84</v>
@@ -4209,13 +4215,13 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
@@ -4267,7 +4273,8 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.7109375" style="5" customWidth="1"/>
-    <col min="5" max="6" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="5" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" style="5" customWidth="1"/>
     <col min="8" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
@@ -4278,7 +4285,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4302,7 +4309,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -4316,16 +4323,16 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>37</v>
@@ -4351,16 +4358,16 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>37</v>
@@ -4386,13 +4393,13 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>22</v>
@@ -4453,23 +4460,23 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>31</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>46</v>
@@ -4512,7 +4519,7 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="32.7109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" style="5" customWidth="1"/>
     <col min="7" max="8" width="22.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="25.7109375" style="5" customWidth="1"/>
@@ -4527,7 +4534,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4551,7 +4558,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -4565,28 +4572,28 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>37</v>
@@ -4612,28 +4619,28 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -4659,10 +4666,10 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>60</v>
@@ -4754,11 +4761,11 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>29</v>
@@ -4773,10 +4780,10 @@
         <v>29</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>46</v>
@@ -4822,7 +4829,8 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="32.7109375" style="5" customWidth="1"/>
-    <col min="3" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="3" max="4" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -4830,7 +4838,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4852,7 +4860,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4860,7 +4868,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -4869,7 +4877,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -4877,7 +4885,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -4886,7 +4894,7 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4894,7 +4902,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4903,7 +4911,7 @@
         <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -4929,13 +4937,13 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>31</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -4965,10 +4973,8 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="32.7109375" style="5" customWidth="1"/>
-    <col min="3" max="5" width="12.7109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="4" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="22.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="25.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4977,7 +4983,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4999,7 +5005,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5007,28 +5013,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5036,28 +5042,28 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5065,7 +5071,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5074,16 +5080,16 @@
         <v>59</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>60</v>
@@ -5124,22 +5130,22 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>108</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I6" s="5"/>
     </row>
@@ -5188,7 +5194,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5212,7 +5218,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
@@ -5229,13 +5235,13 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>135</v>
@@ -5267,13 +5273,13 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>135</v>
@@ -5302,7 +5308,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>60</v>
@@ -5375,20 +5381,20 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>46</v>
@@ -5442,7 +5448,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5464,7 +5470,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5472,16 +5478,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5489,16 +5495,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5506,7 +5512,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5541,7 +5547,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>26</v>
@@ -5580,7 +5586,7 @@
     <col min="5" max="5" width="32.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" style="5" customWidth="1"/>
     <col min="7" max="7" width="16.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="22.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="5" customWidth="1"/>
     <col min="10" max="12" width="12.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="13.7109375" style="5" customWidth="1"/>
@@ -5591,7 +5597,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5615,7 +5621,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
@@ -5629,19 +5635,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>135</v>
@@ -5670,19 +5676,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>135</v>
@@ -5714,7 +5720,7 @@
         <v>84</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>22</v>
@@ -5723,7 +5729,7 @@
         <v>22</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>22</v>
@@ -5790,7 +5796,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -5801,16 +5807,16 @@
         <v>45</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>46</v>
@@ -5869,7 +5875,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5891,7 +5897,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5899,13 +5905,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5913,13 +5919,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5927,13 +5933,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -5956,7 +5962,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="5"/>
     </row>
@@ -6249,7 +6255,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6271,7 +6277,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6279,16 +6285,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6296,16 +6302,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6313,7 +6319,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6348,7 +6354,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>
@@ -6397,7 +6403,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6419,7 +6425,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6427,7 +6433,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6436,16 +6442,16 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6453,7 +6459,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6462,16 +6468,16 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6479,13 +6485,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
@@ -6494,7 +6500,7 @@
         <v>22</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>60</v>
@@ -6532,11 +6538,11 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>27</v>
@@ -6589,7 +6595,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6611,7 +6617,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6619,13 +6625,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6633,13 +6639,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6647,7 +6653,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6676,7 +6682,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
feat(config): G03-P3-B4 author curios and occurrences
</commit_message>
<xml_diff>
--- a/config/generated/templates/Universe.xlsx
+++ b/config/generated/templates/Universe.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1660" uniqueCount="266">
   <si>
     <t>@table</t>
   </si>
@@ -569,7 +569,7 @@
     <t>UniverseCurioState</t>
   </si>
   <si>
-    <t>ff1cd044905089ff</t>
+    <t>d16aad4de9f50377</t>
   </si>
   <si>
     <t>curio_id</t>
@@ -581,6 +581,9 @@
     <t>charges_decimal</t>
   </si>
   <si>
+    <t>charge_parameter_index</t>
+  </si>
+  <si>
     <t>next_state_id</t>
   </si>
   <si>
@@ -603,6 +606,9 @@
   </si>
   <si>
     <t>optional&lt;ref&lt;UniverseCurio.id&gt;&gt;</t>
+  </si>
+  <si>
+    <t>range=0..128</t>
   </si>
   <si>
     <t>UniverseCurioParameter</t>
@@ -3351,7 +3357,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -3359,15 +3365,16 @@
     <col min="4" max="4" width="21.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="28.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" style="5" customWidth="1"/>
-    <col min="7" max="8" width="32.7109375" style="5" customWidth="1"/>
-    <col min="9" max="9" width="31.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="5" customWidth="1"/>
-    <col min="12" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" style="5" customWidth="1"/>
+    <col min="8" max="9" width="32.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="31.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="13" max="15" width="12.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3399,7 +3406,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="24" customHeight="1">
+    <row r="2" spans="1:16" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -3431,22 +3438,25 @@
         <v>181</v>
       </c>
       <c r="K2" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
@@ -3478,22 +3488,25 @@
         <v>181</v>
       </c>
       <c r="K3" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="M3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="O3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="P3" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -3504,25 +3517,25 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>60</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>184</v>
+        <v>21</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>185</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>22</v>
+        <v>186</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>22</v>
@@ -3539,8 +3552,11 @@
       <c r="O4" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="P4" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
@@ -3586,8 +3602,11 @@
       <c r="O5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
@@ -3602,29 +3621,32 @@
       <c r="F6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>187</v>
+      </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="5"/>
+      <c r="K6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>163</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>46</v>
+        <v>163</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="42" customHeight="1">
+      <c r="P6" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
@@ -3642,15 +3664,20 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
       <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Active, Repairing, Fixed" promptTitle="UniverseCurioStateKind enum" prompt="Select a value from the dropdown." sqref="E8:E1007">
       <formula1>"Active,Repairing,Fixed"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 128." promptTitle="Integer range" prompt="Enter an integer from 0 to 128." sqref="G8:G1007">
+      <formula1>0</formula1>
+      <formula2>128</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3922,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3944,7 +3971,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -3952,7 +3979,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -3966,7 +3993,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -3980,7 +4007,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4052,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4076,7 +4103,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4090,13 +4117,13 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>149</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>37</v>
@@ -4122,13 +4149,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>149</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>37</v>
@@ -4285,7 +4312,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4309,7 +4336,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="24" customHeight="1">
@@ -4323,16 +4350,16 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>37</v>
@@ -4358,16 +4385,16 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>37</v>
@@ -4393,7 +4420,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
@@ -4464,10 +4491,10 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>31</v>
@@ -4534,7 +4561,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4558,7 +4585,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -4572,28 +4599,28 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>37</v>
@@ -4619,28 +4646,28 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -4666,7 +4693,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>137</v>
@@ -4761,11 +4788,11 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>29</v>
@@ -4838,7 +4865,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4860,7 +4887,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4868,7 +4895,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -4877,7 +4904,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -4885,7 +4912,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -4894,7 +4921,7 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4902,7 +4929,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -4983,7 +5010,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5005,7 +5032,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5013,28 +5040,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5042,28 +5069,28 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5071,7 +5098,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5139,10 +5166,10 @@
         <v>139</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>139</v>
@@ -5194,7 +5221,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5218,7 +5245,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
@@ -5235,13 +5262,13 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>135</v>
@@ -5273,13 +5300,13 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>135</v>
@@ -5308,7 +5335,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>60</v>
@@ -5448,7 +5475,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5470,7 +5497,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5478,16 +5505,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5495,16 +5522,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5512,7 +5539,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5597,7 +5624,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5621,7 +5648,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
@@ -5635,19 +5662,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>135</v>
@@ -5676,19 +5703,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>135</v>
@@ -5720,7 +5747,7 @@
         <v>84</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>22</v>
@@ -5875,7 +5902,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5897,7 +5924,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5905,13 +5932,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5919,13 +5946,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5933,13 +5960,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -6255,7 +6282,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6277,7 +6304,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6285,16 +6312,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6302,16 +6329,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6319,7 +6346,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6403,7 +6430,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6425,7 +6452,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6433,7 +6460,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6442,16 +6469,16 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>143</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6459,7 +6486,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6468,16 +6495,16 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>143</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6485,13 +6512,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
@@ -6500,7 +6527,7 @@
         <v>22</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>60</v>
@@ -6595,7 +6622,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6617,7 +6644,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6625,7 +6652,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6639,7 +6666,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6653,7 +6680,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>

</xml_diff>